<commit_message>
refactor(sim/config): 配置表双端归拢 + MovementConfig 实例化（技术债 #1/#2/#3 首批）
- demo_tbitem → tbitemconfig / tbmovementconfig：Luban 表拆分归拢，
  GameData/Generated/Lua 三份产物同步，服务端退役 RoomServer/Data/*.json 改读 .bytes（双端同源）
- MovementConfig 从 CombatConfig 静态装载面拆出（技术债 #1 配置实例化首批）；
  SimInputFrame/MovementSystem/EditMode 与 LiteNet.Tests 随动
- scripts/gen-build-hash.py 源集同步新表路径，BuildHash 重跑守卫绿
- 待办总览 7.1/7.2：批次 A（实体分型表）设计入档 + 技术债六项登记
- 排除未纳入：MagicaCloth2 资产线（manifest/ProjectSettings/包本体）、
  训练场相机微调（动画线）、Shell/ 生成器旧路径产物
</commit_message>
<xml_diff>
--- a/Luban/Data/__tables__.xlsx
+++ b/Luban/Data/__tables__.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="144525" fullCalcOnLoad="1"/>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="20.375" customWidth="1" style="2" min="2" max="2"/>
@@ -580,12 +580,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>demo.TbItem</t>
+          <t>TbItemConfig</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>demo.Item</t>
+          <t>ItemConfig</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>#demo.item.xlsx</t>
+          <t>#itemconfig.xlsx</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
@@ -603,14 +603,21 @@
           <t>id</t>
         </is>
       </c>
+      <c r="G4" s="0" t="inlineStr"/>
+      <c r="H4" s="0" t="inlineStr">
+        <is>
+          <t>c,s</t>
+        </is>
+      </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t>demo 道具表</t>
-        </is>
-      </c>
+          <t>道具表（类型 + 刷新/拾取/携带/使用 + 各类型效果数值）</t>
+        </is>
+      </c>
+      <c r="J4" s="0" t="inlineStr"/>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t>demo_tbitem</t>
+          <t>itemconfig</t>
         </is>
       </c>
     </row>
@@ -783,6 +790,55 @@
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>TbMovementConfig</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>MovementConfig</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>#movementconfig.xlsx</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr"/>
+      <c r="H9" s="0" t="inlineStr">
+        <is>
+          <t>c,s</t>
+        </is>
+      </c>
+      <c r="I9" s="0" t="inlineStr">
+        <is>
+          <t>移动数值表（单行：走跑冲/加减速/滑铲/空中/跳跃/钩爪/闪现；消费点 MovementConfig 静态类）</t>
+        </is>
+      </c>
+      <c r="J9" s="0" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>movementconfig</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(l10n): LText 文案表入生成链——#ltext 表源 + Tbltext 生成物 + 表现层 hash 排除
- 表源 #ltext.xlsx（41 键：五页 §8 总表 + 批C 增补，key/zh/en；zh→zh-CN 投射映射归装配批）
- 登记行要点：value_type=TextEntry、index=key（string 主键 map）、group 空（同 tbuiform 判例）
- 实测坑（登记）：Luban 的 #text.xlsx 是其 L10N 家族保留名——文件以该名存在于 Data/ 即
  令 schema 装载抛「TString→TBean」，与登记行无关；表源定名 #ltext.xlsx 避让。
  该版本生成名（bytes/表类/bean/lua）全部派生自输入文件名 ⇒ 产物为 tbltext.bytes/
  Tbltext/cfg.ltext/tbltext.lua，TableLayout 与 DATA_EXCLUDE_NAMES 同批对齐
- gen-build-hash DATA_EXCLUDE_NAMES +tbltext.bytes（纯表现——改文案不得拒进房，
  同 tbuiform 判据）；--check 复算共享常量 ccc7cdb85bc51cba 不变 ✓
- L1 1636/1636 全绿（TableLayout 消费面/表守卫/纪律扫描全过）
- 待办：Unity 导入/重编译 0 错误核证随编辑器恢复后补（本批 .meta 已由编辑器生成）
</commit_message>
<xml_diff>
--- a/Luban/Data/__tables__.xlsx
+++ b/Luban/Data/__tables__.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -333,7 +333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="20.375" customWidth="1" style="2" min="2" max="2"/>
@@ -902,6 +902,51 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>TbText</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>TextEntry</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>#ltext.xlsx</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="G13" s="0" t="n"/>
+      <c r="H13" s="0" t="n"/>
+      <c r="I13" s="0" t="inlineStr">
+        <is>
+          <t>LText 文案表（key→zh/en；BindLocale 数据源——表现层，进 DATA_EXCLUDE_NAMES；表源 #ltext.xlsx）</t>
+        </is>
+      </c>
+      <c r="J13" s="0" t="n"/>
+      <c r="K13" s="0" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>